<commit_message>
* SRS: updated SRS-ED-06 to list 433 MHz as the channel frequency, due to hardware constraints. * Endpoint: implemented application layer command logic. * Gateway: implemented LoRa MAC-switching logic, as well as the API that will be needed for by UART logic. * Overall: added README and UML diagrams
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -133,7 +133,7 @@
     <t xml:space="preserve">SRS-ED-06</t>
   </si>
   <si>
-    <t xml:space="preserve">The LoRa radio shall be configured with: BW=125 kHz, SF=7, CR=4/5, frequency 868.1 MHz (EU868 region), TX power = +14 dBm.</t>
+    <t xml:space="preserve">The LoRa radio shall be configured with: BW=125 kHz, SF=7, CR=4/5, frequency 433 MHz (EU433 region), TX power = +14 dBm.</t>
   </si>
   <si>
     <t xml:space="preserve">Measure RSSI on Gateway side, verify radio parameters in lora_config.h</t>
@@ -1095,64 +1095,68 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1411,713 +1415,713 @@
   <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="5" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G15" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="5" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="7" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="7" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="5" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="5" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G25" s="6" t="s">
+      <c r="G25" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="H25" s="7" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="G27" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="H27" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="5" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2144,437 +2148,440 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="12" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="7" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>255</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="G15" s="14" t="s">
+      <c r="G15" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="I15" s="14" t="s">
+      <c r="I15" s="15" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="7" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="7" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="5" t="s">
         <v>185</v>
       </c>
     </row>
@@ -2603,218 +2610,218 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>235</v>
       </c>
     </row>
@@ -2841,193 +2848,193 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>280</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented telemetry uplink part of UART-MQTT python gateway. Made a few updates to the SRS.
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="SRS" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="276">
   <si>
     <t xml:space="preserve">Software Requirements Specification (SRS) — STM32WL LoRa IoT Gateway</t>
   </si>
@@ -635,7 +635,7 @@
     <t xml:space="preserve">Trigger</t>
   </si>
   <si>
-    <t xml:space="preserve">enddev{N}/sensor/{SensorID}</t>
+    <t xml:space="preserve">enddev{N}/sensor</t>
   </si>
   <si>
     <t xml:space="preserve">EndDevice → Cloud</t>
@@ -644,31 +644,16 @@
     <t xml:space="preserve">Smartphone / Dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">uint32 big-endian (4 bytes) or ASCII decimal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b'\x00\x00\x04\xD2' (=1234)</t>
+    <t xml:space="preserve">2 bytes: SensorID (1B) | SensorValue (1B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b'\x00\x1a' (Button press count=26)</t>
   </si>
   <si>
     <t xml:space="preserve">Reception of LoRa frame TypeID=0x01 by Gateway</t>
   </si>
   <si>
-    <t xml:space="preserve">N=EndDeviceID ; SensorID=0x01 for this project</t>
-  </si>
-  <si>
-    <t xml:space="preserve">enddev1/sensor/1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint32 big-endian decoded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b'\x00\x00\x01\x00' (=256)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LoRa frame TypeID=0x01 SourceID=0x01 SensorID=0x01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concrete topic for EndDevice 1, SensorID 1</t>
+    <t xml:space="preserve">N=EndDeviceID ; SensorID=0x00 for this project</t>
   </si>
   <si>
     <t xml:space="preserve">enddev+/actuator</t>
@@ -790,7 +775,7 @@
 2 s RX window</t>
   </si>
   <si>
-    <t xml:space="preserve">BW=125kHz SF=7 CR=4/5 868.1 MHz</t>
+    <t xml:space="preserve">BW=125kHz SF=7 CR=4/5 433 MHz</t>
   </si>
   <si>
     <t xml:space="preserve">STM32WL Gateway</t>
@@ -840,14 +825,14 @@
     <t xml:space="preserve">Modules: uart_parser, mqtt_client, lora_frame</t>
   </si>
   <si>
-    <t xml:space="preserve">MQTT Broker — HiveMQ</t>
+    <t xml:space="preserve">MQTT Broker — Mosquitto</t>
   </si>
   <si>
     <t xml:space="preserve">Routes messages between Python App and Smartphone</t>
   </si>
   <si>
     <t xml:space="preserve">Public cloud
-broker.hivemq.com:1883</t>
+test.mosquitto.org:1883</t>
   </si>
   <si>
     <t xml:space="preserve">TCP/IP port 1883</t>
@@ -2607,7 +2592,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
@@ -2696,135 +2681,110 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D7" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="E7" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="F8" s="5" t="s">
+      <c r="D8" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="E8" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="F8" s="7" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="H8" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>235</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
@@ -2860,7 +2820,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2872,7 +2832,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2887,22 +2847,22 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>238</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>243</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>9</v>
@@ -2910,54 +2870,54 @@
     </row>
     <row r="4" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>246</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>253</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2965,51 +2925,51 @@
         <v>76</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>260</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>268</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3017,25 +2977,25 @@
         <v>103</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>275</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replaced python bridge app. Gateway: updated RSSI injection to be biased, in accordance with SRS-GW-05
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="SRS" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="278">
   <si>
     <t xml:space="preserve">Software Requirements Specification (SRS) — STM32WL LoRa IoT Gateway</t>
   </si>
@@ -656,19 +656,22 @@
     <t xml:space="preserve">N=EndDeviceID ; SensorID=0x00 for this project</t>
   </si>
   <si>
-    <t xml:space="preserve">enddev+/actuator</t>
+    <t xml:space="preserve">enddev{N}/actuator</t>
   </si>
   <si>
     <t xml:space="preserve">Cloud → EndDevice</t>
   </si>
   <si>
+    <t xml:space="preserve">Dashboard / MQTT Client</t>
+  </si>
+  <si>
     <t xml:space="preserve">2 bytes: ActuatorID (1B) | Cmd (1B)</t>
   </si>
   <si>
     <t xml:space="preserve">b'\x01\x01' (LED1=ON)</t>
   </si>
   <si>
-    <t xml:space="preserve">User action on smartphone app</t>
+    <t xml:space="preserve">User action on dashboard app</t>
   </si>
   <si>
     <t xml:space="preserve">Wildcard + covers all EndDevices</t>
@@ -680,7 +683,7 @@
     <t xml:space="preserve">Smartphone</t>
   </si>
   <si>
-    <t xml:space="preserve">ActuatorID (1B) | Cmd (1B: 0x01=ON 0x00=OFF)</t>
+    <t xml:space="preserve">ActuatorID (1B: 0x01=LED) | Cmd (1B: 0x01=ON 0x00=OFF)</t>
   </si>
   <si>
     <t xml:space="preserve">b'\x01\x01'</t>
@@ -716,16 +719,19 @@
     <t xml:space="preserve">Monitoring Dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">int8 signed ASCII (dBm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b'-85'</t>
+    <t xml:space="preserve">int16 signed integer</t>
   </si>
   <si>
     <t xml:space="preserve">Optional: published on each LoRa reception</t>
   </si>
   <si>
     <t xml:space="preserve">Enables radio link quality monitoring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enddev1/snr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int8 signed integer</t>
   </si>
   <si>
     <t xml:space="preserve">System Architecture — STM32WL LoRa IoT Gateway</t>
@@ -2688,53 +2694,53 @@
         <v>208</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>101</v>
+        <v>209</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>208</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>201</v>
@@ -2746,41 +2752,67 @@
         <v>202</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>-120</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="C9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="E9" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>-5</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H9" s="5" t="s">
         <v>230</v>
       </c>
     </row>
@@ -2820,7 +2852,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2832,7 +2864,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2847,22 +2879,22 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>9</v>
@@ -2870,54 +2902,54 @@
     </row>
     <row r="4" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2925,51 +2957,51 @@
         <v>76</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,25 +3009,25 @@
         <v>103</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated SRS and README.
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="SRS" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="281">
   <si>
     <t xml:space="preserve">Software Requirements Specification (SRS) — STM32WL LoRa IoT Gateway</t>
   </si>
@@ -73,217 +73,220 @@
     <t xml:space="preserve">Analyse the LoRa frame received on the Gateway side: period 5 s ± 200 ms</t>
   </si>
   <si>
+    <t xml:space="preserve">Implemented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulated value via TIM timer or ADC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-ED-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The LoRa uplink packet shall follow the defined 8-byte format: SOF (0xA5) | SourceID (1B) | DestID (1B) | TypeID (1B) | Data (4B big-endian).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capture the raw LoRa frame on the Gateway, decode field by field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SourceID = EndDeviceID ; DestID = GatewayID (0x00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-ED-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The EndDevice shall listen in LoRa RX mode after each transmission (2 s RX window) to receive one valid actuator command packet sent by the Gateway.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send a downlink packet from the Gateway, verify the LED is actuated within 2.5 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RX window enabled via SubGHz_Phy RX callback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-ED-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upon reception of a valid downlink packet (SOF=0xA5, DestID matches own EndDeviceID, TypeID=0x02), the EndDevice shall extract ActuatorID and Data[0] and drive the LED accordingly (Data[0]=0x01 → ON, 0x00 → OFF).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send ON then OFF command, verify LED state with multimeter or oscilloscope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED on GPIO PB11 by default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-ED-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The EndDevice shall send an ACK uplink packet after executing an actuator command: SOF=0xA5 | SourceID=EndDeviceID | DestID=GatewayID | TypeID=0x03 | ActuatorID (1B) | Status (1B: 0x00=OK) | Reserved (2B=0x0000).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEDIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify ACK reception by Gateway and MQTT publication on topic enddev1/ack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TypeID=0x03 reserved for ACK frames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-ED-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The LoRa radio shall be configured with: BW=125 kHz, SF=7, CR=4/5, frequency 433 MHz (EU433 region), TX power = +14 dBm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measure RSSI on Gateway side, verify radio parameters in lora_config.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameters in lora_app.h with justification comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-GW-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gateway FW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The STM32WL Gateway firmware shall receive LoRa uplink packets from EndDevices, validate the SOF (0xA5), and forward the frame to the PC via UART (115200 bps, 8N1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parse 50 consecutive frames on the Python side, verify 0 framing errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UART2 to PC via USB-UART cable (FTDI or ST-Link VCP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-GW-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The UART frame from Gateway to PC shall follow the same 8-byte LoRa format: SOF (0xA5) | SourceID (1B) | DestID (1B) | TypeID (1B) | Data (4B). No additional encapsulation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capture UART stream with serial terminal, decode each field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full transparency: the LoRa frame is forwarded as-is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-GW-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Gateway shall receive 8-byte UART frames from the PC (Python app) and retransmit them as LoRa downlink packets to the EndDevice targeted by the DestID field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send command from Python, verify LoRa TX packet on Gateway (RSSI log)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gateway = bidirectional bridge UART ↔ LoRa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-GW-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Gateway shall filter UART frames received from the PC: SOF ≠ 0xA5 → frame rejected, error counter incremented. No invalid LoRa transmission shall be emitted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inject spurious bytes on UART, verify no unwanted LoRa TX occurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error counter exposed via UART debug command</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-GW-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Gateway shall include the RSSI and SNR of the last received packet in the UART frame sent to the PC, encoded in the reserved bytes when TypeID=0x01: Data[2]=RSSI (signed, dBm offset +200), Data[3]=SNR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify RSSI/SNR fields displayed in the Python dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional if TypeID≠0x01, leave Data[2..3]=0x00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-UART-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UART Gateway↔PC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The UART frame shall be a fixed 8-byte length: SOF (0xA5) | SourceID (1B) | DestID (1B) | TypeID (1B) | Data[0] (1B) | Data[1] (1B) | Data[2] (1B) | Data[3] (1B).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gateway FW / Python</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parse 100 consecutive frames, verify 0 framing errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOF=0xA5 as the sole delimiter — fixed 8-byte frame</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-UART-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The UART link shall operate at 115200 bps, 8 data bits, no parity, 1 stop bit (8N1). The connection shall be established without third-party drivers under Linux (ST-Link VCP or FTDI).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open the COM port, verify frame reception within 100 ms after LoRa TX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USART2 on STM32WL Nucleo: PA2/PA3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-UART-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Python parser shall synchronise on the SOF (0xA5) and read exactly the next 7 bytes. Any frame with missing SOF or incorrect length shall be discarded and increment an invalid frame counter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inject spurious bytes into the UART stream, verify no exception and counter incremented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dedicated serial reader thread with inter-thread queue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-PY-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python Gateway App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Python application shall automatically detect and connect to the STM32WL Gateway UART/VCP port at startup. Identification by STMicroelectronics VID/PID or by scanning available COM ports.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plug in the Gateway, launch the Python app, verify auto-connect within 3 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pyserial.tools.list_ports — VID:0x0483 PID:0x5740</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-PY-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For each UART frame received with TypeID=0x01 (sensor telemetry), the Python app shall publish to the public Mosquitto MQTT broker (test.mosquitto.org:1883) on topic: enddev{SourceID}/sensor with the Sensor ID and Data value (1 byte each).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify MQTT message reception in HiveMQ WebSocket client: correct topic and payload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QoS=0, retain=False ; SensorID = TypeID for v1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-PY-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Python app shall subscribe to the MQTT topic enddev+/actuator (single-level wildcard) on the Mosquitto broker. Upon message reception, it shall build and send an 8-byte UART frame to the Gateway.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publish from dashboard on enddev1/actuator, verify UART frame emitted on serial port</t>
+  </si>
+  <si>
     <t xml:space="preserve">To Do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simulated value via TIM timer or ADC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-ED-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The LoRa uplink packet shall follow the defined 8-byte format: SOF (0xA5) | SourceID (1B) | DestID (1B) | TypeID (1B) | Data (4B big-endian).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capture the raw LoRa frame on the Gateway, decode field by field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SourceID = EndDeviceID ; DestID = GatewayID (0x01)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-ED-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The EndDevice shall listen in LoRa RX mode after each transmission (2 s RX window) to receive actuator command packets sent by the Gateway.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Send a downlink packet from the Gateway, verify the LED is actuated within 2.5 s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RX window enabled via SubGHz_Phy RX callback</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-ED-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upon reception of a valid downlink packet (SOF=0xA5, DestID matches own EndDeviceID, TypeID=0x02), the EndDevice shall extract ActuatorID and Data[0] and drive the LED accordingly (Data[0]=0x01 → ON, 0x00 → OFF).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Send ON then OFF command, verify LED state with multimeter or oscilloscope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LED on GPIO PA5 by default</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-ED-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The EndDevice shall send an ACK uplink packet after executing an actuator command: SOF=0xA5 | SourceID=EndDeviceID | DestID=GatewayID | TypeID=0x03 | ActuatorID (1B) | Status (1B: 0x00=OK) | Reserved (2B=0x0000).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEDIUM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify ACK reception by Gateway and MQTT publication on topic enddev1/ack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TypeID=0x03 reserved for ACK frames</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-ED-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The LoRa radio shall be configured with: BW=125 kHz, SF=7, CR=4/5, frequency 433 MHz (EU433 region), TX power = +14 dBm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Measure RSSI on Gateway side, verify radio parameters in lora_config.h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameters in lora_config.h with justification comments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-GW-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gateway FW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The STM32WL Gateway firmware shall receive LoRa uplink packets from EndDevices, validate the SOF (0xA5), and forward the frame to the PC via UART (115200 bps, 8N1).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parse 50 consecutive frames on the Python side, verify 0 framing errors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART2 to PC via USB-UART cable (FTDI or ST-Link VCP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-GW-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The UART frame from Gateway to PC shall follow the same 8-byte LoRa format: SOF (0xA5) | SourceID (1B) | DestID (1B) | TypeID (1B) | Data (4B). No additional encapsulation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capture UART stream with serial terminal, decode each field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full transparency: the LoRa frame is forwarded as-is</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-GW-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Gateway shall receive 8-byte UART frames from the PC (Python app) and retransmit them as LoRa downlink packets to the EndDevice targeted by the DestID field.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Send command from Python, verify LoRa TX packet on Gateway (RSSI log)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gateway = bidirectional bridge UART ↔ LoRa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-GW-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Gateway shall filter UART frames received from the PC: SOF ≠ 0xA5 → frame rejected, error counter incremented. No invalid LoRa transmission shall be emitted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inject spurious bytes on UART, verify no unwanted LoRa TX occurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error counter exposed via UART debug command</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-GW-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Gateway shall include the RSSI and SNR of the last received packet in the UART frame sent to the PC, encoded in the reserved bytes when TypeID=0x01: Data[2]=RSSI (signed, dBm offset +200), Data[3]=SNR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify RSSI/SNR fields displayed in the Python dashboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional if TypeID≠0x01, leave Data[2..3]=0x00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-UART-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART Gateway↔PC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The UART frame shall be a fixed 8-byte length: SOF (0xA5) | SourceID (1B) | DestID (1B) | TypeID (1B) | Data[0] (1B) | Data[1] (1B) | Data[2] (1B) | Data[3] (1B).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gateway FW / Python</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parse 100 consecutive frames, verify 0 framing errors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOF=0xA5 as the sole delimiter — fixed 8-byte frame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-UART-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The UART link shall operate at 115200 bps, 8 data bits, no parity, 1 stop bit (8N1). The connection shall be established without third-party drivers under Windows 10+ (ST-Link VCP or FTDI).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open the COM port, verify frame reception within 100 ms after LoRa TX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USART2 on STM32WL Nucleo: PA2/PA3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-UART-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Python parser shall synchronise on the SOF (0xA5) and read exactly the next 7 bytes. Any frame with missing SOF or incorrect length shall be discarded and increment an invalid frame counter.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Python</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inject spurious bytes into the UART stream, verify no exception and counter incremented</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dedicated serial reader thread with inter-thread queue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-PY-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Python Gateway App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Python application shall automatically detect and connect to the STM32WL Gateway UART/VCP port at startup. Identification by STMicroelectronics VID/PID or by scanning available COM ports.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plug in the Gateway, launch the Python app, verify auto-connect within 3 s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pyserial.tools.list_ports — VID:0x0483 PID:0x5740</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-PY-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For each UART frame received with TypeID=0x01 (sensor telemetry), the Python app shall publish to the public HiveMQ MQTT broker (broker.hivemq.com:1883) on topic: enddev{SourceID}/sensor/{SensorID} with the Data value (4 bytes big-endian decoded as uint32).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify MQTT message reception in HiveMQ WebSocket client: correct topic and payload</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QoS=0, retain=False ; SensorID = TypeID for v1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-PY-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Python app shall subscribe to the MQTT topic enddev+/actuator (multi-level wildcard) on the HiveMQ broker. Upon message reception, it shall build and send an 8-byte UART frame to the Gateway.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Publish from smartphone on enddev1/actuator, verify UART frame emitted on serial port</t>
   </si>
   <si>
     <t xml:space="preserve">Expected MQTT payload: ActuatorID (1B) | Data (1B)</t>
@@ -719,7 +722,10 @@
     <t xml:space="preserve">Monitoring Dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">int16 signed integer</t>
+    <t xml:space="preserve">int16 signed integer, big-endian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b’\xFF\x88’ = -120</t>
   </si>
   <si>
     <t xml:space="preserve">Optional: published on each LoRa reception</t>
@@ -732,6 +738,9 @@
   </si>
   <si>
     <t xml:space="preserve">int8 signed integer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b’\xFB’ = -5</t>
   </si>
   <si>
     <t xml:space="preserve">System Architecture — STM32WL LoRa IoT Gateway</t>
@@ -1412,7 +1421,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="28"/>
   </cols>
   <sheetData>
@@ -1902,21 +1911,21 @@
         <v>86</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>76</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>72</v>
@@ -1925,24 +1934,24 @@
         <v>14</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>72</v>
@@ -1951,24 +1960,24 @@
         <v>32</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>76</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>72</v>
@@ -1977,76 +1986,76 @@
         <v>32</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>13</v>
@@ -2055,24 +2064,24 @@
         <v>32</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>72</v>
@@ -2081,39 +2090,39 @@
         <v>32</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2148,7 +2157,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2160,7 +2169,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2172,85 +2181,85 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
@@ -2262,25 +2271,25 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>9</v>
@@ -2288,111 +2297,111 @@
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>255</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E12" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>179</v>
-      </c>
       <c r="G12" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -2404,176 +2413,176 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="G17" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>185</v>
-      </c>
       <c r="H17" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2612,7 +2621,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2624,7 +2633,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2636,25 +2645,25 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>9</v>
@@ -2662,158 +2671,158 @@
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>76</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>76</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>76</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>-120</v>
+        <v>229</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>230</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E9" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>-5</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2852,7 +2861,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2864,7 +2873,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2879,22 +2888,22 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>9</v>
@@ -2902,54 +2911,54 @@
     </row>
     <row r="4" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2957,77 +2966,77 @@
         <v>76</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the LED's ActuatorID in the SRS to correspond to the implementation (0x01 -> 0x00).
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -551,7 +551,7 @@
     <t xml:space="preserve">Data[1]=Cmd (ON/OFF), [2..3]=0x00</t>
   </si>
   <si>
-    <t xml:space="preserve">ActuatorID=0x01 → LED</t>
+    <t xml:space="preserve">ActuatorID=0x00 → LED</t>
   </si>
   <si>
     <t xml:space="preserve">0x03</t>
@@ -671,7 +671,7 @@
     <t xml:space="preserve">2 bytes: ActuatorID (1B) | Cmd (1B)</t>
   </si>
   <si>
-    <t xml:space="preserve">b'\x01\x01' (LED1=ON)</t>
+    <t xml:space="preserve">b'\x00\x01' (LED1=ON)</t>
   </si>
   <si>
     <t xml:space="preserve">User action on dashboard app</t>
@@ -689,7 +689,7 @@
     <t xml:space="preserve">ActuatorID (1B: 0x01=LED) | Cmd (1B: 0x01=ON 0x00=OFF)</t>
   </si>
   <si>
-    <t xml:space="preserve">b'\x01\x01'</t>
+    <t xml:space="preserve">b'\x00\x01'</t>
   </si>
   <si>
     <t xml:space="preserve">ON/OFF button on smartphone app</t>
@@ -704,7 +704,7 @@
     <t xml:space="preserve">ActuatorID (1B) | Status (1B: 0x00=OK 0x01=ERR)</t>
   </si>
   <si>
-    <t xml:space="preserve">b'\x01\x00' (LED1 ACK OK)</t>
+    <t xml:space="preserve">b'\x00\x00' (LED1 ACK OK)</t>
   </si>
   <si>
     <t xml:space="preserve">Reception of LoRa frame TypeID=0x03 by Gateway</t>

</xml_diff>

<commit_message>
Fixed conflicts between SRS and python bridge app.
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="SRS" sheetId="1" state="visible" r:id="rId3"/>
@@ -271,7 +271,7 @@
     <t xml:space="preserve">For each UART frame received with TypeID=0x01 (sensor telemetry), the Python app shall publish to the public Mosquitto MQTT broker (test.mosquitto.org:1883) on topic: enddev{SourceID}/sensor with the Sensor ID and Data value (1 byte each).</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify MQTT message reception in HiveMQ WebSocket client: correct topic and payload</t>
+    <t xml:space="preserve">Verify MQTT message reception in test.mosquitto.org client: correct topic and payload</t>
   </si>
   <si>
     <t xml:space="preserve">QoS=0, retain=False ; SensorID = TypeID for v1.0</t>
@@ -286,64 +286,64 @@
     <t xml:space="preserve">Publish from dashboard on enddev1/actuator, verify UART frame emitted on serial port</t>
   </si>
   <si>
+    <t xml:space="preserve">MQTT wildcard normalised to +/actuator (enddev+/actuator is malformed per MQTT v3.1.1 sec 4.7.1); spurious matches filtered by ^enddev(\d+)/actuator$ regex. Subscription re-armed on every reconnect.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-PY-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The actuator command UART frame built by Python shall follow: SOF=0xA5 | SourceID=GatewayID (0x00) | DestID=EndDeviceID (extracted from MQTT topic) | TypeID=0x02 | ActuatorID (1B) | Data[0] (1B) | Reserved (2B=0x00).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capture the UART frame with a serial terminal, validate each field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DestID extracted from enddev{N}/actuator → N converted to byte ; GatewayID=0x00 per firmware (the endpoint sees the command as arriving from the gateway / core network).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-PY-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Python app shall display a timestamped log entry in the console for each processed frame: direction (UP/DOWN), SourceID, DestID, TypeID, Data (hex), MQTT topic published or received.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify presence of all fields in the console log for 10 frames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format: [HH:MM:SS.mmm] DIR SRC→DST TypeID Data MQTT_topic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-PY-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On MQTT disconnection, the app shall attempt automatic reconnection every 5 s with exponential back-off capped at 60 s. On UART disconnection, reconnection shall be attempted every 2 s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cut the network then restore it, verify automatic MQTT reconnection in the log</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use paho-mqtt on_disconnect callback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-MQTT-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smartphone / MQTT Client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The smartphone client (e.g. MQTT Explorer, IoT MQTT Panel) shall subscribe to topic enddev1/sensor/# to receive all telemetry data from EndDevice 1 and display the decoded value in real time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smartphone App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open the app, verify value updated within 10 s after EndDevice LoRa TX</t>
+  </si>
+  <si>
     <t xml:space="preserve">To Do</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected MQTT payload: ActuatorID (1B) | Data (1B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-PY-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The actuator command UART frame built by Python shall follow: SOF=0xA5 | SourceID=GatewayID (0x01) | DestID=EndDeviceID (extracted from MQTT topic) | TypeID=0x02 | ActuatorID (1B) | Data[0] (1B) | Reserved (2B=0x00).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capture the UART frame with a serial terminal, validate each field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DestID extracted from enddev{N}/actuator → N converted to byte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-PY-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Python app shall display a timestamped log entry in the console for each processed frame: direction (UP/DOWN), SourceID, DestID, TypeID, Data (hex), MQTT topic published or received.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify presence of all fields in the console log for 10 frames</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format: [HH:MM:SS.mmm] DIR SRC→DST TypeID Data MQTT_topic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-PY-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On MQTT disconnection, the app shall attempt automatic reconnection every 5 s with exponential back-off capped at 60 s. On UART disconnection, reconnection shall be attempted every 2 s.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cut the network then restore it, verify automatic MQTT reconnection in the log</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use paho-mqtt on_disconnect callback</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-MQTT-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smartphone / MQTT Client</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The smartphone client (e.g. MQTT Explorer, IoT MQTT Panel) shall subscribe to topic enddev1/sensor/# to receive all telemetry data from EndDevice 1 and display the decoded value in real time.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smartphone App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open the app, verify value updated within 10 s after EndDevice LoRa TX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public broker: broker.hivemq.com:1883</t>
+    <t xml:space="preserve">Public broker: test.mosquitto.org:1883</t>
   </si>
   <si>
     <t xml:space="preserve">SRS-MQTT-02</t>
@@ -462,11 +462,11 @@
   <si>
     <t xml:space="preserve">Sender ID
 (0x01=EndDev1
-0x01=Gateway)</t>
+0x00=Gateway)</t>
   </si>
   <si>
     <t xml:space="preserve">Recipient ID
-(0x01=Gateway
+(0x00=Gateway
 0x01=EndDev1)</t>
   </si>
   <si>
@@ -617,7 +617,7 @@
     <t xml:space="preserve">MQTT Topic Mapping — Topics &amp; Payload Format</t>
   </si>
   <si>
-    <t xml:space="preserve">Public broker: broker.hivemq.com:1883  |  QoS=0  |  retain=False</t>
+    <t xml:space="preserve">Public broker: test.mosquitto.org:1883  |  QoS=0  |  retain=False</t>
   </si>
   <si>
     <t xml:space="preserve">MQTT Topic</t>
@@ -1100,63 +1100,63 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1449,7 +1449,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1911,21 +1911,21 @@
         <v>86</v>
       </c>
       <c r="G20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>87</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>76</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>72</v>
@@ -1934,24 +1934,24 @@
         <v>14</v>
       </c>
       <c r="F21" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>72</v>
@@ -1960,24 +1960,24 @@
         <v>32</v>
       </c>
       <c r="F22" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>76</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>72</v>
@@ -1986,36 +1986,36 @@
         <v>32</v>
       </c>
       <c r="F23" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" s="7" t="s">
         <v>99</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>104</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F24" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G24" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>87</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>106</v>
@@ -2026,13 +2026,13 @@
         <v>107</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>108</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>14</v>
@@ -2041,7 +2041,7 @@
         <v>109</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>110</v>
@@ -2067,7 +2067,7 @@
         <v>114</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>115</v>
@@ -2093,7 +2093,7 @@
         <v>118</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>119</v>
@@ -2119,7 +2119,7 @@
         <v>124</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>125</v>
@@ -2179,7 +2179,7 @@
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>128</v>
       </c>
@@ -2269,7 +2269,7 @@
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
         <v>153</v>
       </c>
@@ -2411,7 +2411,7 @@
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
         <v>157</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>159</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>159</v>
@@ -2480,7 +2480,7 @@
         <v>159</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>159</v>
@@ -2506,7 +2506,7 @@
         <v>185</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>159</v>
@@ -2535,7 +2535,7 @@
         <v>185</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>159</v>
@@ -2567,7 +2567,7 @@
         <v>159</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>173</v>
@@ -2643,7 +2643,7 @@
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>195</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
@@ -2883,7 +2883,7 @@
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -3015,7 +3015,7 @@
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>274</v>

</xml_diff>

<commit_message>
`gateway::lora_app.c` unit tests: OnTxDone and OnRxDone tests written and validated.
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="SRS" sheetId="1" state="visible" r:id="rId3"/>
@@ -349,7 +349,7 @@
     <t xml:space="preserve">SRS-MQTT-02</t>
   </si>
   <si>
-    <t xml:space="preserve">The smartphone client shall publish an actuator command on topic enddev1/actuator with payload: ActuatorID (1B hex, e.g. 0x01) | Data (1B hex, e.g. 0x01 for ON). The Python Gateway app shall process this message within 1 s.</t>
+    <t xml:space="preserve">The smartphone client shall publish an actuator command on topic enddev1/actuator with payload: ActuatorID (1B hex, e.g. 0x00) | Data (1B hex, e.g. 0x01 for ON). The Python Gateway app shall process this message within 1 s.</t>
   </si>
   <si>
     <t xml:space="preserve">Publish from smartphone, measure latency until LED actuation on EndDevice</t>
@@ -605,10 +605,10 @@
     <t xml:space="preserve">0xD2</t>
   </si>
   <si>
-    <t xml:space="preserve">CMD LED ON (ActuatorID=0x01), GW→EndDev1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMD LED OFF (ActuatorID=0x01), GW→EndDev1</t>
+    <t xml:space="preserve">CMD LED ON (ActuatorID=0x00), GW→EndDev1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMD LED OFF (ActuatorID=0x00), GW→EndDev1</t>
   </si>
   <si>
     <t xml:space="preserve">ACK LED OK, EndDev1→GW</t>
@@ -1100,63 +1100,63 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>